<commit_message>
feat(F-NAR-019): ATOM-COL.ECO.002-07 L'oiseau en papier de Nina
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-COL.ECO.002-07.xlsx
+++ b/stories/arbres/ATOM-COL.ECO.002-07.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le chien et le linge de Nina</t>
+          <t>L'oiseau en papier de Nina</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>jardin au linge, puis classe</t>
+          <t>cuisine au rayon, classe au coussin vert, puis maison</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Nina, papa, maman, maîtresse</t>
+          <t>Nina, papa, maman</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nina veut raconter le chien brun sous le linge. Le mot est déjà là. Elle lève la main, elle attend, puis elle parle.</t>
+          <t>Un rayon traverse la cuisine. La poussière danse. Sur une aile, un éclat de pli brille. Nina veut montrer l'oiseau en papier, maintenant. Elle tire trop vite : les mots se perdent. À la classe, elle ouvre la bouche trop tôt. Elle refuse de foncer, lève la main, attend, parle du chien. Merci vécu. L'éclat de pli tient sur l'aile.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le fil du jardin est encore mouillé. Un drap blanc danse un peu. Une chaussette rouge se balance. Le linge sent le savon clair. Nina, le doudou sèche aussi. Le chien est dessous, tu vois ? Le chien brun lève le nez. Il renifle le drap. Ses oreilles sont toutes douces. Il veut le doudou. Il sent le savon. Ton oiseau en papier, sur le fil. Nina a accroché l'oiseau. Les ailes sont roses, un peu froissées. Il tourne. Oui. Le vent le tourne. On va à l'école. Tes chaussettes, près du banc. Je glisse tes chaussures. Une, deux. La gauche d'abord. Oui. La gauche d'abord. Le lacet fait un petit nœud. L'oiseau en papier reste ici. Le chien le garde. On marche. Une abeille passe près de la haie. La classe sent la craie. Un oiseau en papier tourne au plafond. La ficelle fait un tout petit bruit. Le coussin vert est à ta place. Au revoir, Nina. Au revoir, maman. On t'attend à la porte, plus tard. En ce moment, Nina s'assoit. Le tissu vert est doux. La craie rose attend dans le bac. Bonjour, Nina. Bonjour. Quel animal aimez-vous ? Nina a une idée. Le chien brun sous le drap. Les oreilles toutes douces. Le mot est déjà là. Elle ouvre un peu la bouche. La maîtresse essuie encore le tableau. La craie fait un petit nuage rose.</t>
+          <t>Un rayon de soleil traverse la cuisine. La poussière danse dans la lumière. Le plancher de bois est tiède. Le tablier de maman sent le savon. Un pied nu touche le bois. La chaleur monte sous le pied, lente. Un fil de poussière va jusqu'au tablier. Un oiseau en papier attend près du sac. Il a des ailes roses, maman. C'est le papier, sous le rayon. Tes chaussettes sont près du banc. Papa glisse les chaussures, une, deux. La gauche d'abord. Oui, la gauche. Le lacet fait un petit nœud. Ton sac est prêt. L'oiseau en papier est dedans. Sur une aile, un éclat de pli brille. Je le vois, papa ! Je veux le montrer, maintenant ! On marche, Nina ? Je le sors ! Nina tire l'oiseau en papier trop vite. L'oiseau en papier glisse, presque. Les mots se cognent à ceux de papa. Personne ne tourne la tête vers elle. Oh. L'éclat de pli tremble, puis tient. Le sourire de Nina s'en va. Dans sa poitrine, ça tape fort. L'envie pousse, puis l'inquiétude. Ça ne veut pas. Ses épaules tombent un peu, lourdes. Papa se met à sa hauteur. Tu veux le montrer ? Oui, papa. Tu mets tes chaussures ? D'accord, maman. Nina glisse un pied, puis l'autre. Le banc est lisse, un peu froid. On marche vers la porte. Le soleil tape sur le chemin. Nina serre le sac contre elle. Il est là, dedans. Oui, dans le sac. Une abeille passe près de la haie. Au revoir, Nina. Au revoir, maman. On t'attend à la porte. En ce moment, Nina s'assoit. Le coussin vert est à sa place. Le tissu vert est doux sous les genoux. La classe sent le papier sec. Ça sent le bois, près des chaises. Une chaise grince près du mur, un peu. Nina pose les genoux sur le tissu. Un oiseau en papier tourne au plafond. La ficelle fait un petit bruit. Nina pose le sac contre le pied. L'oiseau en papier reste dedans. Elle regarde l'oiseau du plafond. Les ailes roses, comme les siennes. La maîtresse parle près du mur. Nina a une idée, très nette. Le chien de la maison est brun. Je veux parler du chien.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le fil du jardin est encore mouillé. Un drap blanc danse un peu. Une chaussette rouge se balance. Le linge sent le savon clair. Nina, le doudou sèche aussi. Le chien est dessous, tu vois ? Le chien brun lève le nez. Il renifle le drap. Ses oreilles sont toutes douces. Il veut le doudou. Il sent le savon. Ton oiseau en papier, sur le fil. Nina a accroché l'oiseau. Les ailes sont roses, un peu froissées. Il tourne. Oui. Le vent le tourne. On va à l'école. Tes chaussettes, près du banc. Je glisse tes chaussures. Une, deux. La gauche d'abord. Oui. La gauche d'abord. Le lacet fait un petit nœud. L'oiseau en papier reste ici. Le chien le garde. On marche. Une abeille passe près de la haie. La classe sent la craie. Un oiseau en papier tourne au plafond. La ficelle fait un tout petit bruit. Le coussin vert est à ta place. Au revoir, Nina. Au revoir, maman. On t'attend à la porte, plus tard. En ce moment, Nina s'assoit. Le tissu vert est doux. La craie rose attend dans le bac. Bonjour, Nina. Bonjour. Quel animal aimez-vous ? Nina a une idée. Le chien brun sous le drap. Les oreilles toutes douces. Le mot est déjà là. Elle ouvre un peu la bouche. La maîtresse essuie encore le tableau. La craie fait un petit nuage rose.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un rayon de soleil traverse la cuisine. La poussière danse dans la lumière. Le plancher de bois est tiède. Le tablier de maman sent le savon. Un pied nu touche le bois. La chaleur monte sous le pied, lente. Un fil de poussière va jusqu'au tablier. Un oiseau en papier attend près du sac. Il a des ailes roses, maman. C'est le papier, sous le rayon. Tes chaussettes sont près du banc. Papa glisse les chaussures, une, deux. La gauche d'abord. Oui, la gauche. Le lacet fait un petit nœud. Ton sac est prêt. L'oiseau en papier est dedans. Sur une aile, un &lt;emphasis level="moderate"&gt;éclat de pli&lt;/emphasis&gt; brille. Je le vois, papa ! Je veux le montrer, maintenant ! On marche, Nina ? Je le sors ! Nina tire l'oiseau en papier trop vite. L'oiseau en papier glisse, presque. Les mots se cognent à ceux de papa. Personne ne tourne la tête vers elle. Oh. L'éclat de pli tremble, puis tient. Le sourire de Nina s'en va. Dans sa poitrine, ça tape fort. L'envie pousse, puis l'inquiétude. Ça ne veut pas. Ses épaules tombent un peu, lourdes. Papa se met à sa hauteur. Tu veux le montrer ? Oui, papa. Tu mets tes chaussures ? D'accord, maman. Nina glisse un pied, puis l'autre. Le banc est lisse, un peu froid. On marche vers la porte. Le soleil tape sur le chemin. Nina serre le sac contre elle. Il est là, dedans. Oui, dans le sac. Une abeille passe près de la haie. Au revoir, Nina. Au revoir, maman. On t'attend à la porte. En ce moment, Nina s'assoit. Le coussin vert est à sa place. Le tissu vert est doux sous les genoux. La classe sent le papier sec. Ça sent le bois, près des chaises. Une chaise grince près du mur, un peu. Nina pose les genoux sur le tissu. Un oiseau en papier tourne au plafond. La ficelle fait un petit bruit. Nina pose le sac contre le pied. L'oiseau en papier reste dedans. Elle regarde l'oiseau du plafond. Les ailes roses, comme les siennes. La maîtresse parle près du mur. Nina a une idée, très nette. Le chien de la maison est brun. Je veux parler du chien.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Delphine arrive en classe. Maman dit au revoir. Delphine s'assoit. La maîtresse pose une question. Delphine a une idée. Elle lève la main. Il faut &lt;emphasis&gt;attendre&lt;/emphasis&gt;. Un camarade parle d'abord. Delphine attend encore. Puis la maîtresse dit : Delphine. C'est ton tour. Delphine parle. Elle dit : le chien est brun. Le soir, maman demande. Delphine dit : j'ai attendu. Puis j'ai parlé. Maman dit : merci. Attendre, puis parler.&lt;/slow&gt; [pause]</t>
+          <t>Un rayon de soleil traverse la cuisine. La poussière danse dans la lumière. Le plancher de bois est tiède. Le tablier de maman sent le savon. Un pied nu touche le bois. La chaleur monte sous le pied, lente. Un fil de poussière va jusqu'au tablier. Un oiseau en papier attend près du sac. Il a des ailes roses, maman. C'est le papier, sous le rayon. Tes chaussettes sont près du banc. Papa glisse les chaussures, une, deux. La gauche d'abord. Oui, la gauche. Le lacet fait un petit nœud. Ton sac est prêt. L'oiseau en papier est dedans. Sur une aile, un &lt;emphasis&gt;éclat de pli&lt;/emphasis&gt; brille. Je le vois, papa ! Je veux le montrer, maintenant ! On marche, Nina ? Je le sors ! Nina tire l'oiseau en papier trop vite. L'oiseau en papier glisse, presque. Les mots se cognent à ceux de papa. Personne ne tourne la tête vers elle. Oh. L'éclat de pli tremble, puis tient. Le sourire de Nina s'en va. Dans sa poitrine, ça tape fort. L'envie pousse, puis l'inquiétude. Ça ne veut pas. Ses épaules tombent un peu, lourdes. Papa se met à sa hauteur. Tu veux le montrer ? Oui, papa. Tu mets tes chaussures ? D'accord, maman. Nina glisse un pied, puis l'autre. Le banc est lisse, un peu froid. On marche vers la porte. Le soleil tape sur le chemin. Nina serre le sac contre elle. Il est là, dedans. Oui, dans le sac. Une abeille passe près de la haie. Au revoir, Nina. Au revoir, maman. On t'attend à la porte. En ce moment, Nina s'assoit. Le coussin vert est à sa place. Le tissu vert est doux sous les genoux. La classe sent le papier sec. Ça sent le bois, près des chaises. Une chaise grince près du mur, un peu. Nina pose les genoux sur le tissu. Un oiseau en papier tourne au plafond. La ficelle fait un petit bruit. Nina pose le sac contre le pied. L'oiseau en papier reste dedans. Elle regarde l'oiseau du plafond. Les ailes roses, comme les siennes. La maîtresse parle près du mur. Nina a une idée, très nette. Le chien de la maison est brun. Je veux parler du chien. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,18 +1246,18 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.28</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>attendre</t>
+          <t>éclat de pli</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1324,65 +1324,86 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_montrer_l_oiseau_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le fil du jardin est encore mouillé.
-narrateur|Un drap blanc danse un peu.
-narrateur|Une chaussette rouge se balance.
-narrateur|Le linge sent le savon clair.
-maman|Nina, le doudou sèche aussi.
-papa|Le chien est dessous, tu vois ?
-narrateur|Le chien brun lève le nez.
-narrateur|Il renifle le drap.
-narrateur|Ses oreilles sont toutes douces.
-enfant-f|Il veut le doudou.
-maman|Il sent le savon.
-papa|Ton oiseau en papier, sur le fil.
-narrateur|Nina a accroché l'oiseau.
-narrateur|Les ailes sont roses, un peu froissées.
-enfant-f|Il tourne.
-papa|Oui.
-papa|Le vent le tourne.
-maman|On va à l'école.
-maman|Tes chaussettes, près du banc.
-papa|Je glisse tes chaussures.
-papa|Une, deux.
+          <t>narrateur|Un rayon de soleil traverse la cuisine.
+narrateur|La poussière danse dans la lumière.
+narrateur|Le plancher de bois est tiède.
+narrateur|Le tablier de maman sent le savon.
+narrateur|Un pied nu touche le bois.
+narrateur|La chaleur monte sous le pied, lente.
+narrateur|Un fil de poussière va jusqu'au tablier.
+narrateur|Un oiseau en papier attend près du sac.
+enfant-f|Il a des ailes roses, maman.
+maman|C'est le papier, sous le rayon.
+papa|Tes chaussettes sont près du banc.
+narrateur|Papa glisse les chaussures, une, deux.
 enfant-f|La gauche d'abord.
-papa|Oui.
-papa|La gauche d'abord.
+papa|Oui, la gauche.
 narrateur|Le lacet fait un petit nœud.
-maman|L'oiseau en papier reste ici.
-enfant-f|Le chien le garde.
-papa|On marche.
+maman|Ton sac est prêt.
+maman|L'oiseau en papier est dedans.
+narrateur|Sur une aile, un éclat de pli brille.
+enfant-f|Je le vois, papa !
+enfant-f|Je veux le montrer, maintenant !
+papa|On marche, Nina ?
+enfant-f|Je le sors !
+narrateur|Nina tire l'oiseau en papier trop vite.
+narrateur|L'oiseau en papier glisse, presque.
+narrateur|Les mots se cognent à ceux de papa.
+narrateur|Personne ne tourne la tête vers elle.
+enfant-f|Oh.
+narrateur|L'éclat de pli tremble, puis tient.
+narrateur|Le sourire de Nina s'en va.
+narrateur|Dans sa poitrine, ça tape fort.
+narrateur|L'envie pousse, puis l'inquiétude.
+enfant-f|Ça ne veut pas.
+narrateur|Ses épaules tombent un peu, lourdes.
+narrateur|Papa se met à sa hauteur.
+papa|Tu veux le montrer ?
+enfant-f|Oui, papa.
+maman|Tu mets tes chaussures ?
+enfant-f|D'accord, maman.
+narrateur|Nina glisse un pied, puis l'autre.
+narrateur|Le banc est lisse, un peu froid.
+papa|On marche vers la porte.
+narrateur|Le soleil tape sur le chemin.
+narrateur|Nina serre le sac contre elle.
+enfant-f|Il est là, dedans.
+papa|Oui, dans le sac.
 narrateur|Une abeille passe près de la haie.
-narrateur|La classe sent la craie.
-narrateur|Un oiseau en papier tourne au plafond.
-narrateur|La ficelle fait un tout petit bruit.
-maman|Le coussin vert est à ta place.
 maman|Au revoir, Nina.
 enfant-f|Au revoir, maman.
-papa|On t'attend à la porte, plus tard.
+papa|On t'attend à la porte.
 narrateur|En ce moment, Nina s'assoit.
-narrateur|Le tissu vert est doux.
-narrateur|La craie rose attend dans le bac.
-maitresse|Bonjour, Nina.
-enfant-f|Bonjour.
-maitresse|Quel animal aimez-vous ?
-narrateur|Nina a une idée.
-narrateur|Le chien brun sous le drap.
-narrateur|Les oreilles toutes douces.
-narrateur|Le mot est déjà là.
-narrateur|Elle ouvre un peu la bouche.
-narrateur|La maîtresse essuie encore le tableau.
-narrateur|La craie fait un petit nuage rose.</t>
+narrateur|Le coussin vert est à sa place.
+narrateur|Le tissu vert est doux sous les genoux.
+narrateur|La classe sent le papier sec.
+narrateur|Ça sent le bois, près des chaises.
+narrateur|Une chaise grince près du mur, un peu.
+narrateur|Nina pose les genoux sur le tissu.
+narrateur|Un oiseau en papier tourne au plafond.
+narrateur|La ficelle fait un petit bruit.
+narrateur|Nina pose le sac contre le pied.
+narrateur|L'oiseau en papier reste dedans.
+narrateur|Elle regarde l'oiseau du plafond.
+narrateur|Les ailes roses, comme les siennes.
+narrateur|La maîtresse parle près du mur.
+narrateur|Nina a une idée, très nette.
+narrateur|Le chien de la maison est brun.
+enfant-f|Je veux parler du chien.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>chien_bonjour,linge,pas</t>
+          <t>rayon,chaussure,porte</t>
         </is>
       </c>
     </row>
@@ -1414,12 +1435,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Nina veut parler. Que fait-elle d'abord ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Nina veut &lt;emphasis level="moderate"&gt;parler&lt;/emphasis&gt;. Que fait-elle d'abord ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Delphine veut parler. Que fait-elle d'abord ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Nina veut &lt;emphasis&gt;parler&lt;/emphasis&gt;. Que fait-elle d'abord ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1482,7 +1503,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1490,10 +1511,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.4</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1508,34 +1529,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>parler</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1544,13 +1569,13 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1560,7 +1585,7 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=elle_attend_puis_parle; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1593,17 +1618,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Nina lève la main. Sa main reste haute. Elle attend. L'oiseau du plafond tourne encore. Nina le suit des yeux. Sa main ne descend pas. Nina. C'est toi. Tu peux parler. Le chien est brun. Il était sous le linge. Ses oreilles sont douces. Sous le drap blanc ? Oui. Il sentait le savon. Merci, Nina. Un grain de craie rose est tombé. Il brille dans la lumière.</t>
+          <t>Nina ouvre la bouche trop vite. Mon chien est brun ! Un camarade parle, près du coussin. Le chat est noir. Les deux voix se mélangent dans l'air. Oh. Le sourire de Nina ne revient pas. Nina refuse de foncer, cette fois. Elle referme la bouche, un instant. Elle lève la main, près du coussin. Sa main reste en l'air. Le camarade finit sa phrase, loin. Un autre mot arrive, plus loin. Nina garde la main haute, sans bouger. Nina attend que le silence arrive. Elle ouvre un peu le sac. Sur l'aile, l'éclat de pli brille. Je peux dire quelque chose ? La classe tourne un peu la tête. Le chien est brun. Il a les oreilles douces. Elle pose l'oiseau près du coussin. Les ailes roses regardent le plafond. Plus tard, la porte s'ouvre. Te voilà, Nina. Le sac sent le papier. Nina pose le sac près du banc. J'ai parlé du chien. Il a les oreilles douces. Merci, Nina. Papa a entendu toute la phrase. Tu veux voir le chien ? Oui, maman. Le ventre de Nina se desserre.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Nina lève la main. Sa main reste haute. Elle attend. L'oiseau du plafond tourne encore. Nina le suit des yeux. Sa main ne descend pas. Nina. C'est toi. Tu peux parler. Le chien est brun. Il était sous le linge. Ses oreilles sont douces. Sous le drap blanc ? Oui. Il sentait le savon. Merci, Nina. Un grain de craie rose est tombé. Il brille dans la lumière.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina ouvre la bouche trop vite. Mon chien est brun ! Un camarade parle, près du coussin. Le chat est noir. Les deux voix se mélangent dans l'air. Oh. Le sourire de Nina ne revient pas. Nina refuse de foncer, cette fois. Elle referme la bouche, un instant. Elle lève la main, près du coussin. Sa main reste en l'air. Le camarade finit sa phrase, loin. Un autre mot arrive, plus loin. Nina garde la main haute, sans bouger. Nina attend que le &lt;emphasis level="moderate"&gt;silence&lt;/emphasis&gt; arrive. Elle ouvre un peu le sac. Sur l'aile, l'éclat de pli brille. Je peux dire quelque chose ? La classe tourne un peu la tête. Le chien est brun. Il a les oreilles douces. Elle pose l'oiseau près du coussin. Les ailes roses regardent le plafond. Plus tard, la porte s'ouvre. Te voilà, Nina. Le sac sent le papier. Nina pose le sac près du banc. J'ai parlé du chien. Il a les oreilles douces. Merci, Nina. Papa a entendu toute la phrase. Tu veux voir le chien ? Oui, maman. Le ventre de Nina se desserre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Delphine a levé la main. Elle a attendu. &lt;emphasis&gt;puis&lt;/emphasis&gt; elle a parlé. C'était son tour.&lt;/slow&gt; [pause]</t>
+          <t>Nina ouvre la bouche trop vite. Mon chien est brun ! Un camarade parle, près du coussin. Le chat est noir. Les deux voix se mélangent dans l'air. Oh. Le sourire de Nina ne revient pas. Nina refuse de foncer, cette fois. Elle referme la bouche, un instant. Elle lève la main, près du coussin. Sa main reste en l'air. Le camarade finit sa phrase, loin. Un autre mot arrive, plus loin. Nina garde la main haute, sans bouger. Nina attend que le &lt;emphasis&gt;silence&lt;/emphasis&gt; arrive. Elle ouvre un peu le sac. Sur l'aile, l'éclat de pli brille. Je peux dire quelque chose ? La classe tourne un peu la tête. Le chien est brun. Il a les oreilles douces. Elle pose l'oiseau près du coussin. Les ailes roses regardent le plafond. Plus tard, la porte s'ouvre. Te voilà, Nina. Le sac sent le papier. Nina pose le sac près du banc. J'ai parlé du chien. Il a les oreilles douces. Merci, Nina. Papa a entendu toute la phrase. Tu veux voir le chien ? Oui, maman. Le ventre de Nina se desserre. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1650,18 +1675,18 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.28</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1684,30 +1709,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>puis</t>
+          <t>silence</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1716,10 +1741,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1728,33 +1753,54 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_leve_la_main_puis_on_l_entend; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Nina lève la main.
-narrateur|Sa main reste haute.
-narrateur|Elle attend.
-narrateur|L'oiseau du plafond tourne encore.
-narrateur|Nina le suit des yeux.
-narrateur|Sa main ne descend pas.
-maitresse|Nina.
-maitresse|C'est toi.
-maitresse|Tu peux parler.
+          <t>narrateur|Nina ouvre la bouche trop vite.
+enfant-f|Mon chien est brun !
+narrateur|Un camarade parle, près du coussin.
+copain|Le chat est noir.
+narrateur|Les deux voix se mélangent dans l'air.
+enfant-f|Oh.
+narrateur|Le sourire de Nina ne revient pas.
+narrateur|Nina refuse de foncer, cette fois.
+narrateur|Elle referme la bouche, un instant.
+narrateur|Elle lève la main, près du coussin.
+narrateur|Sa main reste en l'air.
+narrateur|Le camarade finit sa phrase, loin.
+narrateur|Un autre mot arrive, plus loin.
+narrateur|Nina garde la main haute, sans bouger.
+narrateur|Nina attend que le silence arrive.
+narrateur|Elle ouvre un peu le sac.
+narrateur|Sur l'aile, l'éclat de pli brille.
+enfant-f|Je peux dire quelque chose ?
+narrateur|La classe tourne un peu la tête.
 enfant-f|Le chien est brun.
-enfant-f|Il était sous le linge.
-enfant-f|Ses oreilles sont douces.
-maitresse|Sous le drap blanc ?
-enfant-f|Oui.
-enfant-f|Il sentait le savon.
-maitresse|Merci, Nina.
-narrateur|Un grain de craie rose est tombé.
-narrateur|Il brille dans la lumière.</t>
+enfant-f|Il a les oreilles douces.
+narrateur|Elle pose l'oiseau près du coussin.
+narrateur|Les ailes roses regardent le plafond.
+narrateur|Plus tard, la porte s'ouvre.
+maman|Te voilà, Nina.
+papa|Le sac sent le papier.
+narrateur|Nina pose le sac près du banc.
+enfant-f|J'ai parlé du chien.
+enfant-f|Il a les oreilles douces.
+papa|Merci, Nina.
+narrateur|Papa a entendu toute la phrase.
+maman|Tu veux voir le chien ?
+enfant-f|Oui, maman.
+narrateur|Le ventre de Nina se desserre.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>coussin,porte</t>
         </is>
       </c>
     </row>
@@ -1781,17 +1827,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, Nina range son cartable. L'oiseau de la classe tourne encore. La porte s'ouvre. Tu as passé un bon moment ? J'ai parlé du chien. Il était sous le linge. Le chien du jardin ? Oui, papa. Ses oreilles sont douces. On rentre. Le soleil suit leurs pas. Une chaussette rouge sèche encore. Le plancher de la maison est tiède. Le chien brun vient tout près. Tes oreilles sont douces. Il t'a reconnue. Le doudou est sec, maintenant. Nina pose sa main sur le chien. Le chien ferme un peu les yeux. Une goutte tombe du drap. Elle fait un petit rond.</t>
+          <t>Le chien brun vient tout près. Nina veut tout montrer, d'un coup. Elle prend l'oiseau en papier. Regarde, les ailes ! Elle déplie l'aile trop vite. Le papier craque sous les doigts, un peu. L'aile s'ouvre trop, d'un coup. Ça tombe ! Nina veut foncer, d'un coup. Nina refuse de foncer, cette fois. Ses épaules se serrent un peu. Ça tape fort, dans sa poitrine. Personne ne dit la suite à voix haute. Elle regarde l'oiseau en papier. Elle écoute la cuisine, un instant. La poussière danse dans le rayon. Le pli de l'aile est trop ouvert. Comme ce matin ? Tu le vois, toi ? Non, plus sur l'aile. Nina plie l'aile, sans se presser. Il est là. Sur cette aile ? Oui, sur ce pli. L'éclat de pli revient, sur l'aile. Le chien, Nina ? Oui. Elle s'assoit près du chien. Le chien pose le nez tout près. Les oreilles sont chaudes, un peu. C'est doux.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, Nina range son cartable. L'oiseau de la classe tourne encore. La porte s'ouvre. Tu as passé un bon moment ? J'ai parlé du chien. Il était sous le linge. Le chien du jardin ? Oui, papa. Ses oreilles sont douces. On rentre. Le soleil suit leurs pas. Une chaussette rouge sèche encore. Le plancher de la maison est tiède. Le chien brun vient tout près. Tes oreilles sont douces. Il t'a reconnue. Le doudou est sec, maintenant. Nina pose sa main sur le chien. Le chien ferme un peu les yeux. Une goutte tombe du drap. Elle fait un petit rond.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Le chien brun vient tout près. Nina veut tout montrer, d'un coup. Elle prend l'oiseau en papier. Regarde, les ailes ! Elle déplie l'aile trop vite. Le papier craque sous les doigts, un peu. L'aile s'ouvre trop, d'un coup. Ça tombe ! Nina veut foncer, d'un coup. Nina refuse de foncer, cette fois. Ses épaules se serrent un peu. Ça tape fort, dans sa poitrine. Personne ne dit la suite à voix haute. Elle regarde l'oiseau en papier. Elle écoute la cuisine, un instant. La poussière danse dans le rayon. Le pli de l'aile est trop ouvert. Comme ce matin ? Tu le vois, toi ? Non, plus sur l'aile. Nina plie l'aile, sans se presser. Il est là. Sur cette aile ? Oui, sur ce pli. L'&lt;emphasis level="moderate"&gt;éclat de pli&lt;/emphasis&gt; revient, sur l'aile. Le chien, Nina ? Oui. Elle s'assoit près du chien. Le chien pose le nez tout près. Les oreilles sont chaudes, un peu. C'est doux.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Delphine range son cartable. Maman l'attend à la porte.&lt;/slow&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Le chien brun vient tout près. Nina veut tout montrer, d'un coup. Elle prend l'oiseau en papier. Regarde, les ailes ! Elle déplie l'aile trop vite. Le papier craque sous les doigts, un peu. L'aile s'ouvre trop, d'un coup. Ça tombe ! Nina veut foncer, d'un coup. Nina refuse de foncer, cette fois. Ses épaules se serrent un peu. Ça tape fort, dans sa poitrine. Personne ne dit la suite à voix haute. Elle regarde l'oiseau en papier. Elle écoute la cuisine, un instant. La poussière danse dans le rayon. Le pli de l'aile est trop ouvert. Comme ce matin ? Tu le vois, toi ? Non, plus sur l'aile. Nina plie l'aile, sans se presser. Il est là. Sur cette aile ? Oui, sur ce pli. L'&lt;emphasis&gt;éclat de pli&lt;/emphasis&gt; revient, sur l'aile. Le chien, Nina ? Oui. Elle s'assoit près du chien. Le chien pose le nez tout près. Les oreilles sont chaudes, un peu. C'est doux.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1838,30 +1884,34 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>134</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.93</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.28</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AE5" s="2" t="inlineStr"/>
+          <t>-2st</t>
+        </is>
+      </c>
+      <c r="AE5" s="2" t="inlineStr">
+        <is>
+          <t>low-pitch</t>
+        </is>
+      </c>
       <c r="AF5" s="2" t="inlineStr">
         <is>
           <t>medium</t>
@@ -1870,28 +1920,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de pli</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>520</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>300</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>tense</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1900,49 +1954,63 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.93</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.93</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
       </c>
       <c r="AT5" s="2" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=obstacle; intention=alerter_sans_effrayer; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_retrouve_l_eclat; tempo=resserré; sourire=aucun; respiration=retenue</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Plus tard, Nina range son cartable.
-narrateur|L'oiseau de la classe tourne encore.
-narrateur|La porte s'ouvre.
-maman|Tu as passé un bon moment ?
-enfant-f|J'ai parlé du chien.
-enfant-f|Il était sous le linge.
-papa|Le chien du jardin ?
-enfant-f|Oui, papa.
-enfant-f|Ses oreilles sont douces.
-maman|On rentre.
-narrateur|Le soleil suit leurs pas.
-narrateur|Une chaussette rouge sèche encore.
-narrateur|Le plancher de la maison est tiède.
-narrateur|Le chien brun vient tout près.
-enfant-f|Tes oreilles sont douces.
-papa|Il t'a reconnue.
-maman|Le doudou est sec, maintenant.
-narrateur|Nina pose sa main sur le chien.
-narrateur|Le chien ferme un peu les yeux.
-narrateur|Une goutte tombe du drap.
-narrateur|Elle fait un petit rond.</t>
+          <t>narrateur|Le chien brun vient tout près.
+narrateur|Nina veut tout montrer, d'un coup.
+narrateur|Elle prend l'oiseau en papier.
+enfant-f|Regarde, les ailes !
+narrateur|Elle déplie l'aile trop vite.
+narrateur|Le papier craque sous les doigts, un peu.
+narrateur|L'aile s'ouvre trop, d'un coup.
+enfant-f|Ça tombe !
+narrateur|Nina veut foncer, d'un coup.
+narrateur|Nina refuse de foncer, cette fois.
+narrateur|Ses épaules se serrent un peu.
+narrateur|Ça tape fort, dans sa poitrine.
+narrateur|Personne ne dit la suite à voix haute.
+narrateur|Elle regarde l'oiseau en papier.
+narrateur|Elle écoute la cuisine, un instant.
+narrateur|La poussière danse dans le rayon.
+narrateur|Le pli de l'aile est trop ouvert.
+enfant-f|Comme ce matin ?
+papa|Tu le vois, toi ?
+enfant-f|Non, plus sur l'aile.
+narrateur|Nina plie l'aile, sans se presser.
+enfant-f|Il est là.
+papa|Sur cette aile ?
+enfant-f|Oui, sur ce pli.
+narrateur|L'éclat de pli revient, sur l'aile.
+maman|Le chien, Nina ?
+enfant-f|Oui.
+narrateur|Elle s'assoit près du chien.
+narrateur|Le chien pose le nez tout près.
+narrateur|Les oreilles sont chaudes, un peu.
+enfant-f|C'est doux.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>chien_bonjour,pas</t>
+          <t>chien_bonjour,papier</t>
         </is>
       </c>
     </row>
@@ -1969,17 +2037,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le drap blanc ne danse plus. Nina pose sa main sur le chien. Les oreilles étaient douces. Bonne soirée, ma grande.</t>
+          <t>L'oiseau en papier attend près du banc. Le rayon reste dans la cuisine. L'éclat est là, papa. Tu le vois sur le pli ? Oui, papa. On est bien, ici. Le tablier de maman sent le savon. Le plancher de bois est tiède. On m'a entendue. On t'a entendue, Nina. Oui, maman. Nina pose la joue près des ailes. Le papier est sec, un peu rêche. C'est froid. Le chien ferme un peu les yeux. L'éclat de pli tient sur l'aile.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le drap blanc ne danse plus. Nina pose sa main sur le chien. Les oreilles étaient douces. Bonne soirée, ma grande.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;L'oiseau en papier attend près du banc. Le rayon reste dans la cuisine. L'éclat est là, papa. Tu le vois sur le pli ? Oui, papa. On est bien, ici. Le tablier de maman sent le savon. Le plancher de bois est tiède. On m'a entendue. On t'a entendue, Nina. Oui, maman. Nina pose la joue près des ailes. Le papier est sec, un peu rêche. C'est froid. Le chien ferme un peu les yeux. L'&lt;emphasis level="moderate"&gt;éclat de pli&lt;/emphasis&gt; tient sur l'aile.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'oiseau en papier attend près du banc. Le rayon reste dans la cuisine. L'éclat est là, papa. Tu le vois sur le pli ? Oui, papa. On est bien, ici. Le tablier de maman sent le savon. Le plancher de bois est tiède. On m'a entendue. On t'a entendue, Nina. Oui, maman. Nina pose la joue près des ailes. Le papier est sec, un peu rêche. C'est froid. Le chien ferme un peu les yeux. L'&lt;emphasis&gt;éclat de pli&lt;/emphasis&gt; tient sur l'aile.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2026,7 +2094,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2034,10 +2102,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.36</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2046,12 +2114,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2060,17 +2128,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de pli</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>380</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2079,11 +2151,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2092,27 +2164,48 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_l_aile; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le drap blanc ne danse plus.
-narrateur|Nina pose sa main sur le chien.
-papa|Les oreilles étaient douces.
-maman|Bonne soirée, ma grande.</t>
+          <t>narrateur|L'oiseau en papier attend près du banc.
+narrateur|Le rayon reste dans la cuisine.
+enfant-f|L'éclat est là, papa.
+papa|Tu le vois sur le pli ?
+enfant-f|Oui, papa.
+maman|On est bien, ici.
+narrateur|Le tablier de maman sent le savon.
+narrateur|Le plancher de bois est tiède.
+enfant-f|On m'a entendue.
+maman|On t'a entendue, Nina.
+enfant-f|Oui, maman.
+narrateur|Nina pose la joue près des ailes.
+narrateur|Le papier est sec, un peu rêche.
+enfant-f|C'est froid.
+narrateur|Le chien ferme un peu les yeux.
+narrateur|L'éclat de pli tient sur l'aile.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>chien_bonjour</t>
         </is>
       </c>
     </row>
@@ -2133,7 +2226,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2218,6 +2311,13 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>